<commit_message>
Tuan09/TH07/tao file excel lưu kết quả cuối của 2 model DT va LR
</commit_message>
<xml_diff>
--- a/eda/ket_qua/ketquacacmohinh.xlsx
+++ b/eda/ket_qua/ketquacacmohinh.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ai-project\eda\ket_qua\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2860F53B-B6EB-40FF-8C02-D4EB5515F6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB4BF26-A7AE-4A2A-9602-794BAB961586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="13">
   <si>
     <t>Validation Accuracy</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>LR</t>
+  </si>
+  <si>
+    <t>Kết quả train khi đã xử lí dữ liệu và chỉnh sửa mô hình</t>
   </si>
 </sst>
 </file>
@@ -413,7 +416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -424,9 +427,13 @@
     <col min="6" max="6" width="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="3.21875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>9</v>
       </c>
@@ -438,8 +445,19 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
+      <c r="L1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -467,8 +485,35 @@
       <c r="I2" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="L2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -496,8 +541,35 @@
       <c r="I3">
         <v>0.5859872611464968</v>
       </c>
+      <c r="L3" t="s">
+        <v>10</v>
+      </c>
+      <c r="M3">
+        <v>0.8125</v>
+      </c>
+      <c r="N3">
+        <v>0.71179039301310043</v>
+      </c>
+      <c r="O3">
+        <v>0.7032844164919636</v>
+      </c>
+      <c r="P3">
+        <v>68</v>
+      </c>
+      <c r="Q3">
+        <v>55</v>
+      </c>
+      <c r="R3">
+        <v>11</v>
+      </c>
+      <c r="S3">
+        <v>95</v>
+      </c>
+      <c r="T3">
+        <v>0.67326732673267331</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -525,10 +597,38 @@
       <c r="I4">
         <v>0.61538461538461542</v>
       </c>
+      <c r="L4" t="s">
+        <v>11</v>
+      </c>
+      <c r="M4">
+        <v>0.76249999999999996</v>
+      </c>
+      <c r="N4">
+        <v>0.73799126637554591</v>
+      </c>
+      <c r="O4">
+        <v>0.75199161425576511</v>
+      </c>
+      <c r="P4">
+        <v>54</v>
+      </c>
+      <c r="Q4">
+        <v>35</v>
+      </c>
+      <c r="R4">
+        <v>25</v>
+      </c>
+      <c r="S4">
+        <v>115</v>
+      </c>
+      <c r="T4">
+        <v>0.6428571428571429</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="L1:T1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>